<commit_message>
Updates the random EV-parameter distribution to take demand into account, avoids infeasibility due to too small maximum battery capacity.
</commit_message>
<xml_diff>
--- a/data_preparation/standard_ev_battery_data.xlsx
+++ b/data_preparation/standard_ev_battery_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\V2G-QUESTS\data_preparation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\V2G-QUESTS-PSOM\data_preparation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AAB0AE2-057D-4648-9192-D30B4E287B3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F961BAE-C92F-4194-BAEE-55E78C748695}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="40930" yWindow="4000" windowWidth="28800" windowHeight="15240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="72850" yWindow="2170" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -484,7 +484,7 @@
         <v>0.98</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.5">
@@ -510,7 +510,7 @@
         <v>0.98</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.5">
@@ -536,7 +536,7 @@
         <v>0.98</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.5">
@@ -562,7 +562,7 @@
         <v>0.98</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.5">
@@ -588,7 +588,7 @@
         <v>0.98</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.5">
@@ -614,7 +614,7 @@
         <v>0.98</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.5">
@@ -640,7 +640,7 @@
         <v>0.98</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.5">
@@ -666,7 +666,7 @@
         <v>0.98</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.5">
@@ -692,7 +692,7 @@
         <v>0.98</v>
       </c>
       <c r="H10">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.5">
@@ -718,7 +718,7 @@
         <v>0.98</v>
       </c>
       <c r="H11">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add EV/V2G charging options and internal uncontrolled charging calculation. Update battery/EV and V2G discharge formulations and optimize model building using predefined dictionaries.
</commit_message>
<xml_diff>
--- a/data_preparation/standard_ev_battery_data.xlsx
+++ b/data_preparation/standard_ev_battery_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\V2G-QUESTS-PSOM\data_preparation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\V2G-QUESTS\data_preparation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F961BAE-C92F-4194-BAEE-55E78C748695}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEA844FA-1B02-4513-B87A-5E6E0997F5B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="72850" yWindow="2170" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34450" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -484,7 +484,7 @@
         <v>0.98</v>
       </c>
       <c r="H2">
-        <v>0.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.5">
@@ -510,7 +510,7 @@
         <v>0.98</v>
       </c>
       <c r="H3">
-        <v>0.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.5">
@@ -536,7 +536,7 @@
         <v>0.98</v>
       </c>
       <c r="H4">
-        <v>0.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.5">
@@ -562,7 +562,7 @@
         <v>0.98</v>
       </c>
       <c r="H5">
-        <v>0.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.5">
@@ -588,7 +588,7 @@
         <v>0.98</v>
       </c>
       <c r="H6">
-        <v>0.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.5">
@@ -599,10 +599,10 @@
         <v>12</v>
       </c>
       <c r="C7">
-        <v>9.5000000000000001E-2</v>
+        <v>0.123</v>
       </c>
       <c r="D7">
-        <v>1.0999999999999999E-2</v>
+        <v>2.1999999999999999E-2</v>
       </c>
       <c r="E7">
         <v>3.5999999999999999E-3</v>
@@ -614,7 +614,7 @@
         <v>0.98</v>
       </c>
       <c r="H7">
-        <v>0.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.5">
@@ -625,10 +625,10 @@
         <v>16</v>
       </c>
       <c r="C8">
-        <v>6.0499999999999998E-2</v>
+        <v>0.11799999999999999</v>
       </c>
       <c r="D8">
-        <v>7.0000000000000001E-3</v>
+        <v>1.0999999999999999E-2</v>
       </c>
       <c r="E8">
         <v>2.2000000000000001E-3</v>
@@ -640,7 +640,7 @@
         <v>0.98</v>
       </c>
       <c r="H8">
-        <v>0.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.5">
@@ -651,10 +651,10 @@
         <v>15</v>
       </c>
       <c r="C9">
-        <v>5.0299999999999997E-2</v>
+        <v>7.0999999999999994E-2</v>
       </c>
       <c r="D9">
-        <v>1.0999999999999999E-2</v>
+        <v>2.1999999999999999E-2</v>
       </c>
       <c r="E9">
         <v>2.2000000000000001E-3</v>
@@ -666,7 +666,7 @@
         <v>0.98</v>
       </c>
       <c r="H9">
-        <v>0.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.5">
@@ -677,10 +677,10 @@
         <v>11</v>
       </c>
       <c r="C10">
-        <v>4.4899999999999995E-2</v>
+        <v>0.04</v>
       </c>
       <c r="D10">
-        <v>7.0000000000000001E-3</v>
+        <v>1.0999999999999999E-2</v>
       </c>
       <c r="E10">
         <v>3.3E-3</v>
@@ -692,7 +692,7 @@
         <v>0.98</v>
       </c>
       <c r="H10">
-        <v>0.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.5">
@@ -703,10 +703,10 @@
         <v>10</v>
       </c>
       <c r="C11">
-        <v>1.3800000000000002E-2</v>
+        <v>2.1299999999999999E-2</v>
       </c>
       <c r="D11">
-        <v>3.7000000000000002E-3</v>
+        <v>1.0999999999999999E-2</v>
       </c>
       <c r="E11">
         <v>1.5E-3</v>
@@ -718,7 +718,7 @@
         <v>0.98</v>
       </c>
       <c r="H11">
-        <v>0.2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>